<commit_message>
Publish complete SLD coverage and 500 kV IBT view
</commit_message>
<xml_diff>
--- a/samples/ss_bdgsel_nubrg_ingest.xlsx
+++ b/samples/ss_bdgsel_nubrg_ingest.xlsx
@@ -767,7 +767,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">

</xml_diff>